<commit_message>
Correct submodule for 20260223 version of ICTVdatabase repo
</commit_message>
<xml_diff>
--- a/VMR_MSL40v2_20260223/errors.xlsx
+++ b/VMR_MSL40v2_20260223/errors.xlsx
@@ -568,7 +568,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Read 4 rows from file ICTVdatabase_20260122/data/taxonomy_genome_coverage.utf8.txt</t>
+          <t>Read 4 rows from file ICTVdatabase_20260223/data/taxonomy_genome_coverage.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -604,7 +604,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Read 14 rows from file ICTVdatabase_20260122/data/taxonomy_molecule.utf8.txt</t>
+          <t>Read 14 rows from file ICTVdatabase_20260223/data/taxonomy_molecule.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -628,7 +628,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Read 27 rows from file ICTVdatabase_20260122/data/taxonomy_host_source.utf8.txt</t>
+          <t>Read 27 rows from file ICTVdatabase_20260223/data/taxonomy_host_source.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -664,7 +664,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Read 4 rows from file ICTVdatabase_20260122/data/taxonomy_genome_coverage.utf8.txt</t>
+          <t>Read 4 rows from file ICTVdatabase_20260223/data/taxonomy_genome_coverage.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -700,7 +700,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Read 14 rows from file ICTVdatabase_20260122/data/taxonomy_molecule.utf8.txt</t>
+          <t>Read 14 rows from file ICTVdatabase_20260223/data/taxonomy_molecule.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -724,7 +724,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Read 27 rows from file ICTVdatabase_20260122/data/taxonomy_host_source.utf8.txt</t>
+          <t>Read 27 rows from file ICTVdatabase_20260223/data/taxonomy_host_source.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1828,7 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Read 17930 rows from file ICTVdatabase_20260122/data/vmr_export.utf8.txt</t>
+          <t>Read 17930 rows from file ICTVdatabase_20260223/data/vmr_export.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -2284,7 +2284,7 @@
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Read 40 rows from file ICTVdatabase_20260122/data/taxonomy_toc.utf8.txt</t>
+          <t>Read 40 rows from file ICTVdatabase_20260223/data/taxonomy_toc.utf8.txt</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Wrote workbook with 8 worksheet(s) to VMR_MSL40.v2.20260122.editor.xlsx</t>
+          <t>Wrote workbook with 8 worksheet(s) to VMR_MSL40.v2.20260223.editor.xlsx</t>
         </is>
       </c>
     </row>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Wrote 4 worksheet(s) to public file VMR_MSL40.v2.20260122.xlsx</t>
+          <t>Wrote 4 worksheet(s) to public file VMR_MSL40.v2.20260223.xlsx</t>
         </is>
       </c>
     </row>

</xml_diff>